<commit_message>
Update to use UserLogin as Student ID for matching HKDSE/IB results
- Change first column from English Name to UserLogin (Student ID)
- Update data loading to recognize UserLogin as primary key
- Improve matching logic for HKDSE/IB data
- Update sample file to use UserLogin column
- Update documentation to reflect UserLogin as Student ID
- Randomize sample data scores for more realistic distribution
</commit_message>
<xml_diff>
--- a/sample_files/sample_eclass_data.xlsx
+++ b/sample_files/sample_eclass_data.xlsx
@@ -425,158 +425,148 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD11"/>
+  <dimension ref="A1:AB11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Student_ID</t>
+          <t>UserLogin</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>English_Name</t>
+          <t>English_Term1</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>English_Term1</t>
+          <t>English_Term2</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>English_Term2</t>
+          <t>English_Term3</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>English_Term3</t>
+          <t>Chinese_Term1</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Chinese_Term1</t>
+          <t>Chinese_Term2</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Chinese_Term2</t>
+          <t>Chinese_Term3</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Chinese_Term3</t>
+          <t>Mathematics_Term1</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Mathematics_Term1</t>
+          <t>Mathematics_Term2</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Mathematics_Term2</t>
+          <t>Mathematics_Term3</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Mathematics_Term3</t>
+          <t>Science_Term1</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Science_Term1</t>
+          <t>Science_Term2</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Science_Term2</t>
+          <t>Science_Term3</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Science_Term3</t>
+          <t>History_Term1</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>History_Term1</t>
+          <t>History_Term2</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>History_Term2</t>
+          <t>History_Term3</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>History_Term3</t>
+          <t>Geography_Term1</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Geography_Term1</t>
+          <t>Geography_Term2</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>Geography_Term2</t>
+          <t>Geography_Term3</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>Geography_Term3</t>
+          <t>Physics_Term1</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>Physics_Term1</t>
+          <t>Physics_Term2</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>Physics_Term2</t>
+          <t>Physics_Term3</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>Physics_Term3</t>
+          <t>Chemistry_Term1</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>Chemistry_Term1</t>
+          <t>Chemistry_Term2</t>
         </is>
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>Chemistry_Term2</t>
+          <t>Chemistry_Term3</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
         <is>
-          <t>Chemistry_Term3</t>
+          <t>Biology_Term1</t>
         </is>
       </c>
       <c r="AA1" s="1" t="inlineStr">
         <is>
-          <t>Biology_Term1</t>
+          <t>Biology_Term2</t>
         </is>
       </c>
       <c r="AB1" s="1" t="inlineStr">
         <is>
-          <t>Biology_Term2</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
           <t>Biology_Term3</t>
-        </is>
-      </c>
-      <c r="AD1" s="1" t="inlineStr">
-        <is>
-          <t>Average_Score</t>
         </is>
       </c>
     </row>
@@ -586,94 +576,86 @@
           <t>STU001</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>STU001</t>
-        </is>
+      <c r="B2" t="n">
+        <v>73</v>
       </c>
       <c r="C2" t="n">
+        <v>82</v>
+      </c>
+      <c r="D2" t="n">
+        <v>80</v>
+      </c>
+      <c r="E2" t="n">
+        <v>60</v>
+      </c>
+      <c r="F2" t="n">
+        <v>69</v>
+      </c>
+      <c r="G2" t="n">
+        <v>85</v>
+      </c>
+      <c r="H2" t="n">
+        <v>74</v>
+      </c>
+      <c r="I2" t="n">
+        <v>82</v>
+      </c>
+      <c r="J2" t="n">
+        <v>100</v>
+      </c>
+      <c r="K2" t="n">
+        <v>61</v>
+      </c>
+      <c r="L2" t="n">
+        <v>81</v>
+      </c>
+      <c r="M2" t="n">
+        <v>69</v>
+      </c>
+      <c r="N2" t="n">
+        <v>70</v>
+      </c>
+      <c r="O2" t="n">
+        <v>67</v>
+      </c>
+      <c r="P2" t="n">
+        <v>68</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>76</v>
+      </c>
+      <c r="R2" t="n">
+        <v>69</v>
+      </c>
+      <c r="S2" t="n">
         <v>75</v>
       </c>
-      <c r="D2" t="n">
-        <v>78</v>
-      </c>
-      <c r="E2" t="n">
-        <v>80</v>
-      </c>
-      <c r="F2" t="n">
-        <v>80</v>
-      </c>
-      <c r="G2" t="n">
-        <v>82</v>
-      </c>
-      <c r="H2" t="n">
+      <c r="T2" t="n">
+        <v>62</v>
+      </c>
+      <c r="U2" t="n">
+        <v>72</v>
+      </c>
+      <c r="V2" t="n">
+        <v>83</v>
+      </c>
+      <c r="W2" t="n">
         <v>85</v>
       </c>
-      <c r="I2" t="n">
+      <c r="X2" t="n">
+        <v>86</v>
+      </c>
+      <c r="Y2" t="n">
         <v>88</v>
       </c>
-      <c r="J2" t="n">
-        <v>90</v>
-      </c>
-      <c r="K2" t="n">
-        <v>92</v>
-      </c>
-      <c r="L2" t="n">
-        <v>82</v>
-      </c>
-      <c r="M2" t="n">
-        <v>84</v>
-      </c>
-      <c r="N2" t="n">
-        <v>86</v>
-      </c>
-      <c r="O2" t="n">
-        <v>78</v>
-      </c>
-      <c r="P2" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>82</v>
-      </c>
-      <c r="R2" t="n">
-        <v>80</v>
-      </c>
-      <c r="S2" t="n">
-        <v>82</v>
-      </c>
-      <c r="T2" t="n">
-        <v>84</v>
-      </c>
-      <c r="U2" t="n">
-        <v>85</v>
-      </c>
-      <c r="V2" t="n">
-        <v>87</v>
-      </c>
-      <c r="W2" t="n">
-        <v>89</v>
-      </c>
-      <c r="X2" t="n">
-        <v>83</v>
-      </c>
-      <c r="Y2" t="n">
-        <v>85</v>
-      </c>
       <c r="Z2" t="n">
-        <v>87</v>
+        <v>67</v>
       </c>
       <c r="AA2" t="n">
-        <v>81</v>
+        <v>70</v>
       </c>
       <c r="AB2" t="n">
-        <v>83</v>
-      </c>
-      <c r="AC2" t="n">
-        <v>85</v>
-      </c>
-      <c r="AD2" t="n">
-        <v>82.3</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3">
@@ -682,94 +664,86 @@
           <t>STU002</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>STU002</t>
-        </is>
+      <c r="B3" t="n">
+        <v>68</v>
       </c>
       <c r="C3" t="n">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="D3" t="n">
-        <v>85</v>
+        <v>63</v>
       </c>
       <c r="E3" t="n">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="F3" t="n">
+        <v>66</v>
+      </c>
+      <c r="G3" t="n">
+        <v>72</v>
+      </c>
+      <c r="H3" t="n">
         <v>78</v>
       </c>
-      <c r="G3" t="n">
-        <v>80</v>
-      </c>
-      <c r="H3" t="n">
-        <v>83</v>
-      </c>
       <c r="I3" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="J3" t="n">
-        <v>87</v>
+        <v>65</v>
       </c>
       <c r="K3" t="n">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="L3" t="n">
-        <v>79</v>
+        <v>55</v>
       </c>
       <c r="M3" t="n">
-        <v>81</v>
+        <v>64</v>
       </c>
       <c r="N3" t="n">
-        <v>83</v>
+        <v>46</v>
       </c>
       <c r="O3" t="n">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="P3" t="n">
-        <v>83</v>
+        <v>63</v>
       </c>
       <c r="Q3" t="n">
-        <v>85</v>
+        <v>70</v>
       </c>
       <c r="R3" t="n">
-        <v>83</v>
+        <v>72</v>
       </c>
       <c r="S3" t="n">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="T3" t="n">
-        <v>87</v>
+        <v>50</v>
       </c>
       <c r="U3" t="n">
-        <v>80</v>
+        <v>62</v>
       </c>
       <c r="V3" t="n">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="W3" t="n">
-        <v>84</v>
+        <v>65</v>
       </c>
       <c r="X3" t="n">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="Y3" t="n">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="Z3" t="n">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="AA3" t="n">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="AB3" t="n">
-        <v>81</v>
-      </c>
-      <c r="AC3" t="n">
-        <v>83</v>
-      </c>
-      <c r="AD3" t="n">
-        <v>82.7</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4">
@@ -778,94 +752,86 @@
           <t>STU003</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>STU003</t>
-        </is>
+      <c r="B4" t="n">
+        <v>65</v>
       </c>
       <c r="C4" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D4" t="n">
+        <v>77</v>
+      </c>
+      <c r="E4" t="n">
+        <v>71</v>
+      </c>
+      <c r="F4" t="n">
+        <v>73</v>
+      </c>
+      <c r="G4" t="n">
+        <v>75</v>
+      </c>
+      <c r="H4" t="n">
+        <v>88</v>
+      </c>
+      <c r="I4" t="n">
+        <v>85</v>
+      </c>
+      <c r="J4" t="n">
+        <v>86</v>
+      </c>
+      <c r="K4" t="n">
+        <v>72</v>
+      </c>
+      <c r="L4" t="n">
+        <v>58</v>
+      </c>
+      <c r="M4" t="n">
+        <v>69</v>
+      </c>
+      <c r="N4" t="n">
+        <v>61</v>
+      </c>
+      <c r="O4" t="n">
+        <v>74</v>
+      </c>
+      <c r="P4" t="n">
+        <v>73</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>90</v>
+      </c>
+      <c r="R4" t="n">
+        <v>73</v>
+      </c>
+      <c r="S4" t="n">
+        <v>84</v>
+      </c>
+      <c r="T4" t="n">
+        <v>66</v>
+      </c>
+      <c r="U4" t="n">
+        <v>72</v>
+      </c>
+      <c r="V4" t="n">
+        <v>82</v>
+      </c>
+      <c r="W4" t="n">
+        <v>78</v>
+      </c>
+      <c r="X4" t="n">
+        <v>86</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>83</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>77</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>75</v>
+      </c>
+      <c r="AB4" t="n">
         <v>70</v>
-      </c>
-      <c r="E4" t="n">
-        <v>72</v>
-      </c>
-      <c r="F4" t="n">
-        <v>72</v>
-      </c>
-      <c r="G4" t="n">
-        <v>74</v>
-      </c>
-      <c r="H4" t="n">
-        <v>77</v>
-      </c>
-      <c r="I4" t="n">
-        <v>70</v>
-      </c>
-      <c r="J4" t="n">
-        <v>72</v>
-      </c>
-      <c r="K4" t="n">
-        <v>74</v>
-      </c>
-      <c r="L4" t="n">
-        <v>75</v>
-      </c>
-      <c r="M4" t="n">
-        <v>77</v>
-      </c>
-      <c r="N4" t="n">
-        <v>79</v>
-      </c>
-      <c r="O4" t="n">
-        <v>68</v>
-      </c>
-      <c r="P4" t="n">
-        <v>70</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>72</v>
-      </c>
-      <c r="R4" t="n">
-        <v>72</v>
-      </c>
-      <c r="S4" t="n">
-        <v>74</v>
-      </c>
-      <c r="T4" t="n">
-        <v>76</v>
-      </c>
-      <c r="U4" t="n">
-        <v>73</v>
-      </c>
-      <c r="V4" t="n">
-        <v>75</v>
-      </c>
-      <c r="W4" t="n">
-        <v>77</v>
-      </c>
-      <c r="X4" t="n">
-        <v>70</v>
-      </c>
-      <c r="Y4" t="n">
-        <v>72</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>74</v>
-      </c>
-      <c r="AA4" t="n">
-        <v>74</v>
-      </c>
-      <c r="AB4" t="n">
-        <v>76</v>
-      </c>
-      <c r="AC4" t="n">
-        <v>78</v>
-      </c>
-      <c r="AD4" t="n">
-        <v>73.5</v>
       </c>
     </row>
     <row r="5">
@@ -874,94 +840,86 @@
           <t>STU004</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>STU004</t>
-        </is>
+      <c r="B5" t="n">
+        <v>84</v>
       </c>
       <c r="C5" t="n">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="D5" t="n">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="E5" t="n">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="F5" t="n">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="G5" t="n">
+        <v>95</v>
+      </c>
+      <c r="H5" t="n">
+        <v>96</v>
+      </c>
+      <c r="I5" t="n">
+        <v>100</v>
+      </c>
+      <c r="J5" t="n">
+        <v>100</v>
+      </c>
+      <c r="K5" t="n">
+        <v>74</v>
+      </c>
+      <c r="L5" t="n">
+        <v>86</v>
+      </c>
+      <c r="M5" t="n">
+        <v>75</v>
+      </c>
+      <c r="N5" t="n">
+        <v>77</v>
+      </c>
+      <c r="O5" t="n">
+        <v>67</v>
+      </c>
+      <c r="P5" t="n">
+        <v>86</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>84</v>
+      </c>
+      <c r="R5" t="n">
+        <v>82</v>
+      </c>
+      <c r="S5" t="n">
         <v>87</v>
       </c>
-      <c r="H5" t="n">
-        <v>90</v>
-      </c>
-      <c r="I5" t="n">
-        <v>92</v>
-      </c>
-      <c r="J5" t="n">
-        <v>94</v>
-      </c>
-      <c r="K5" t="n">
-        <v>96</v>
-      </c>
-      <c r="L5" t="n">
-        <v>88</v>
-      </c>
-      <c r="M5" t="n">
-        <v>90</v>
-      </c>
-      <c r="N5" t="n">
-        <v>92</v>
-      </c>
-      <c r="O5" t="n">
-        <v>85</v>
-      </c>
-      <c r="P5" t="n">
+      <c r="T5" t="n">
         <v>87</v>
       </c>
-      <c r="Q5" t="n">
-        <v>89</v>
-      </c>
-      <c r="R5" t="n">
-        <v>87</v>
-      </c>
-      <c r="S5" t="n">
-        <v>89</v>
-      </c>
-      <c r="T5" t="n">
-        <v>91</v>
-      </c>
       <c r="U5" t="n">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="V5" t="n">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="W5" t="n">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="X5" t="n">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="Y5" t="n">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="Z5" t="n">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="AA5" t="n">
-        <v>86</v>
+        <v>66</v>
       </c>
       <c r="AB5" t="n">
-        <v>88</v>
-      </c>
-      <c r="AC5" t="n">
-        <v>90</v>
-      </c>
-      <c r="AD5" t="n">
-        <v>89.8</v>
+        <v>84</v>
       </c>
     </row>
     <row r="6">
@@ -970,94 +928,86 @@
           <t>STU005</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>STU005</t>
-        </is>
+      <c r="B6" t="n">
+        <v>69</v>
       </c>
       <c r="C6" t="n">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="D6" t="n">
         <v>76</v>
       </c>
       <c r="E6" t="n">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="F6" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="G6" t="n">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="H6" t="n">
-        <v>81</v>
+        <v>66</v>
       </c>
       <c r="I6" t="n">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="J6" t="n">
-        <v>82</v>
+        <v>69</v>
       </c>
       <c r="K6" t="n">
-        <v>84</v>
+        <v>68</v>
       </c>
       <c r="L6" t="n">
-        <v>77</v>
+        <v>51</v>
       </c>
       <c r="M6" t="n">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="N6" t="n">
-        <v>81</v>
+        <v>48</v>
       </c>
       <c r="O6" t="n">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="P6" t="n">
-        <v>76</v>
+        <v>61</v>
       </c>
       <c r="Q6" t="n">
         <v>78</v>
       </c>
       <c r="R6" t="n">
-        <v>79</v>
+        <v>56</v>
       </c>
       <c r="S6" t="n">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="T6" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="U6" t="n">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="V6" t="n">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="W6" t="n">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="X6" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="Y6" t="n">
         <v>77</v>
       </c>
       <c r="Z6" t="n">
-        <v>79</v>
+        <v>59</v>
       </c>
       <c r="AA6" t="n">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="AB6" t="n">
-        <v>78</v>
-      </c>
-      <c r="AC6" t="n">
-        <v>80</v>
-      </c>
-      <c r="AD6" t="n">
-        <v>78.59999999999999</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7">
@@ -1066,94 +1016,86 @@
           <t>STU006</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>STU006</t>
-        </is>
+      <c r="B7" t="n">
+        <v>64</v>
       </c>
       <c r="C7" t="n">
-        <v>85</v>
+        <v>60</v>
       </c>
       <c r="D7" t="n">
-        <v>87</v>
+        <v>67</v>
       </c>
       <c r="E7" t="n">
-        <v>89</v>
+        <v>73</v>
       </c>
       <c r="F7" t="n">
-        <v>82</v>
+        <v>59</v>
       </c>
       <c r="G7" t="n">
-        <v>84</v>
+        <v>59</v>
       </c>
       <c r="H7" t="n">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="I7" t="n">
-        <v>90</v>
+        <v>65</v>
       </c>
       <c r="J7" t="n">
-        <v>92</v>
+        <v>64</v>
       </c>
       <c r="K7" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="L7" t="n">
-        <v>85</v>
+        <v>62</v>
       </c>
       <c r="M7" t="n">
-        <v>87</v>
+        <v>57</v>
       </c>
       <c r="N7" t="n">
-        <v>89</v>
+        <v>70</v>
       </c>
       <c r="O7" t="n">
-        <v>83</v>
+        <v>57</v>
       </c>
       <c r="P7" t="n">
-        <v>85</v>
+        <v>59</v>
       </c>
       <c r="Q7" t="n">
-        <v>87</v>
+        <v>73</v>
       </c>
       <c r="R7" t="n">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="S7" t="n">
-        <v>88</v>
+        <v>64</v>
       </c>
       <c r="T7" t="n">
-        <v>90</v>
+        <v>56</v>
       </c>
       <c r="U7" t="n">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="V7" t="n">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="W7" t="n">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="X7" t="n">
-        <v>86</v>
+        <v>70</v>
       </c>
       <c r="Y7" t="n">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="Z7" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="AA7" t="n">
-        <v>84</v>
+        <v>63</v>
       </c>
       <c r="AB7" t="n">
-        <v>86</v>
-      </c>
-      <c r="AC7" t="n">
-        <v>88</v>
-      </c>
-      <c r="AD7" t="n">
-        <v>87.2</v>
+        <v>63</v>
       </c>
     </row>
     <row r="8">
@@ -1162,94 +1104,86 @@
           <t>STU007</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>STU007</t>
-        </is>
+      <c r="B8" t="n">
+        <v>100</v>
       </c>
       <c r="C8" t="n">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="D8" t="n">
+        <v>97</v>
+      </c>
+      <c r="E8" t="n">
+        <v>94</v>
+      </c>
+      <c r="F8" t="n">
+        <v>90</v>
+      </c>
+      <c r="G8" t="n">
+        <v>85</v>
+      </c>
+      <c r="H8" t="n">
+        <v>96</v>
+      </c>
+      <c r="I8" t="n">
+        <v>91</v>
+      </c>
+      <c r="J8" t="n">
+        <v>100</v>
+      </c>
+      <c r="K8" t="n">
+        <v>94</v>
+      </c>
+      <c r="L8" t="n">
         <v>81</v>
       </c>
-      <c r="E8" t="n">
+      <c r="M8" t="n">
+        <v>95</v>
+      </c>
+      <c r="N8" t="n">
+        <v>74</v>
+      </c>
+      <c r="O8" t="n">
+        <v>74</v>
+      </c>
+      <c r="P8" t="n">
+        <v>89</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>82</v>
+      </c>
+      <c r="R8" t="n">
+        <v>100</v>
+      </c>
+      <c r="S8" t="n">
+        <v>98</v>
+      </c>
+      <c r="T8" t="n">
+        <v>82</v>
+      </c>
+      <c r="U8" t="n">
+        <v>70</v>
+      </c>
+      <c r="V8" t="n">
+        <v>73</v>
+      </c>
+      <c r="W8" t="n">
+        <v>100</v>
+      </c>
+      <c r="X8" t="n">
+        <v>76</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>100</v>
+      </c>
+      <c r="Z8" t="n">
         <v>84</v>
       </c>
-      <c r="F8" t="n">
-        <v>79</v>
-      </c>
-      <c r="G8" t="n">
-        <v>81</v>
-      </c>
-      <c r="H8" t="n">
-        <v>84</v>
-      </c>
-      <c r="I8" t="n">
-        <v>83</v>
-      </c>
-      <c r="J8" t="n">
-        <v>85</v>
-      </c>
-      <c r="K8" t="n">
-        <v>87</v>
-      </c>
-      <c r="L8" t="n">
-        <v>80</v>
-      </c>
-      <c r="M8" t="n">
-        <v>82</v>
-      </c>
-      <c r="N8" t="n">
-        <v>84</v>
-      </c>
-      <c r="O8" t="n">
-        <v>77</v>
-      </c>
-      <c r="P8" t="n">
-        <v>79</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>81</v>
-      </c>
-      <c r="R8" t="n">
-        <v>79</v>
-      </c>
-      <c r="S8" t="n">
-        <v>81</v>
-      </c>
-      <c r="T8" t="n">
-        <v>83</v>
-      </c>
-      <c r="U8" t="n">
-        <v>82</v>
-      </c>
-      <c r="V8" t="n">
-        <v>84</v>
-      </c>
-      <c r="W8" t="n">
-        <v>86</v>
-      </c>
-      <c r="X8" t="n">
-        <v>79</v>
-      </c>
-      <c r="Y8" t="n">
-        <v>81</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>83</v>
-      </c>
       <c r="AA8" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="AB8" t="n">
-        <v>80</v>
-      </c>
-      <c r="AC8" t="n">
-        <v>82</v>
-      </c>
-      <c r="AD8" t="n">
-        <v>81.40000000000001</v>
+        <v>90</v>
       </c>
     </row>
     <row r="9">
@@ -1258,94 +1192,86 @@
           <t>STU008</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>STU008</t>
-        </is>
+      <c r="B9" t="n">
+        <v>76</v>
       </c>
       <c r="C9" t="n">
-        <v>72</v>
+        <v>89</v>
       </c>
       <c r="D9" t="n">
         <v>75</v>
       </c>
       <c r="E9" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F9" t="n">
-        <v>74</v>
+        <v>94</v>
       </c>
       <c r="G9" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H9" t="n">
+        <v>90</v>
+      </c>
+      <c r="I9" t="n">
+        <v>90</v>
+      </c>
+      <c r="J9" t="n">
+        <v>81</v>
+      </c>
+      <c r="K9" t="n">
+        <v>75</v>
+      </c>
+      <c r="L9" t="n">
+        <v>78</v>
+      </c>
+      <c r="M9" t="n">
+        <v>69</v>
+      </c>
+      <c r="N9" t="n">
+        <v>67</v>
+      </c>
+      <c r="O9" t="n">
+        <v>78</v>
+      </c>
+      <c r="P9" t="n">
+        <v>82</v>
+      </c>
+      <c r="Q9" t="n">
         <v>79</v>
       </c>
-      <c r="I9" t="n">
-        <v>75</v>
-      </c>
-      <c r="J9" t="n">
-        <v>77</v>
-      </c>
-      <c r="K9" t="n">
-        <v>79</v>
-      </c>
-      <c r="L9" t="n">
-        <v>73</v>
-      </c>
-      <c r="M9" t="n">
-        <v>75</v>
-      </c>
-      <c r="N9" t="n">
-        <v>77</v>
-      </c>
-      <c r="O9" t="n">
-        <v>71</v>
-      </c>
-      <c r="P9" t="n">
-        <v>73</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>75</v>
-      </c>
       <c r="R9" t="n">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="S9" t="n">
-        <v>75</v>
+        <v>95</v>
       </c>
       <c r="T9" t="n">
-        <v>77</v>
+        <v>96</v>
       </c>
       <c r="U9" t="n">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="V9" t="n">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="W9" t="n">
+        <v>88</v>
+      </c>
+      <c r="X9" t="n">
+        <v>100</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>90</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>66</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>66</v>
+      </c>
+      <c r="AB9" t="n">
         <v>80</v>
-      </c>
-      <c r="X9" t="n">
-        <v>73</v>
-      </c>
-      <c r="Y9" t="n">
-        <v>75</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>77</v>
-      </c>
-      <c r="AA9" t="n">
-        <v>72</v>
-      </c>
-      <c r="AB9" t="n">
-        <v>74</v>
-      </c>
-      <c r="AC9" t="n">
-        <v>76</v>
-      </c>
-      <c r="AD9" t="n">
-        <v>75.2</v>
       </c>
     </row>
     <row r="10">
@@ -1354,94 +1280,86 @@
           <t>STU009</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>STU009</t>
-        </is>
+      <c r="B10" t="n">
+        <v>57</v>
       </c>
       <c r="C10" t="n">
-        <v>88</v>
+        <v>68</v>
       </c>
       <c r="D10" t="n">
-        <v>90</v>
+        <v>71</v>
       </c>
       <c r="E10" t="n">
-        <v>92</v>
+        <v>56</v>
       </c>
       <c r="F10" t="n">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="G10" t="n">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="H10" t="n">
-        <v>91</v>
+        <v>75</v>
       </c>
       <c r="I10" t="n">
-        <v>93</v>
+        <v>76</v>
       </c>
       <c r="J10" t="n">
-        <v>95</v>
+        <v>69</v>
       </c>
       <c r="K10" t="n">
-        <v>97</v>
+        <v>61</v>
       </c>
       <c r="L10" t="n">
-        <v>89</v>
+        <v>53</v>
       </c>
       <c r="M10" t="n">
-        <v>91</v>
+        <v>63</v>
       </c>
       <c r="N10" t="n">
-        <v>93</v>
+        <v>64</v>
       </c>
       <c r="O10" t="n">
-        <v>87</v>
+        <v>59</v>
       </c>
       <c r="P10" t="n">
-        <v>89</v>
+        <v>62</v>
       </c>
       <c r="Q10" t="n">
-        <v>91</v>
+        <v>60</v>
       </c>
       <c r="R10" t="n">
-        <v>88</v>
+        <v>59</v>
       </c>
       <c r="S10" t="n">
-        <v>90</v>
+        <v>66</v>
       </c>
       <c r="T10" t="n">
-        <v>92</v>
+        <v>50</v>
       </c>
       <c r="U10" t="n">
-        <v>91</v>
+        <v>66</v>
       </c>
       <c r="V10" t="n">
-        <v>93</v>
+        <v>71</v>
       </c>
       <c r="W10" t="n">
-        <v>95</v>
+        <v>65</v>
       </c>
       <c r="X10" t="n">
-        <v>89</v>
+        <v>73</v>
       </c>
       <c r="Y10" t="n">
-        <v>91</v>
+        <v>69</v>
       </c>
       <c r="Z10" t="n">
-        <v>93</v>
+        <v>72</v>
       </c>
       <c r="AA10" t="n">
-        <v>87</v>
+        <v>59</v>
       </c>
       <c r="AB10" t="n">
-        <v>89</v>
-      </c>
-      <c r="AC10" t="n">
-        <v>91</v>
-      </c>
-      <c r="AD10" t="n">
-        <v>90.59999999999999</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11">
@@ -1450,94 +1368,86 @@
           <t>STU010</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>STU010</t>
-        </is>
+      <c r="B11" t="n">
+        <v>55</v>
       </c>
       <c r="C11" t="n">
+        <v>78</v>
+      </c>
+      <c r="D11" t="n">
+        <v>77</v>
+      </c>
+      <c r="E11" t="n">
         <v>80</v>
       </c>
-      <c r="D11" t="n">
-        <v>83</v>
-      </c>
-      <c r="E11" t="n">
+      <c r="F11" t="n">
+        <v>76</v>
+      </c>
+      <c r="G11" t="n">
+        <v>80</v>
+      </c>
+      <c r="H11" t="n">
+        <v>81</v>
+      </c>
+      <c r="I11" t="n">
+        <v>91</v>
+      </c>
+      <c r="J11" t="n">
         <v>85</v>
       </c>
-      <c r="F11" t="n">
-        <v>81</v>
-      </c>
-      <c r="G11" t="n">
-        <v>83</v>
-      </c>
-      <c r="H11" t="n">
-        <v>86</v>
-      </c>
-      <c r="I11" t="n">
-        <v>87</v>
-      </c>
-      <c r="J11" t="n">
+      <c r="K11" t="n">
+        <v>65</v>
+      </c>
+      <c r="L11" t="n">
+        <v>67</v>
+      </c>
+      <c r="M11" t="n">
+        <v>68</v>
+      </c>
+      <c r="N11" t="n">
+        <v>65</v>
+      </c>
+      <c r="O11" t="n">
+        <v>75</v>
+      </c>
+      <c r="P11" t="n">
+        <v>69</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>76</v>
+      </c>
+      <c r="R11" t="n">
+        <v>77</v>
+      </c>
+      <c r="S11" t="n">
         <v>89</v>
       </c>
-      <c r="K11" t="n">
-        <v>91</v>
-      </c>
-      <c r="L11" t="n">
-        <v>82</v>
-      </c>
-      <c r="M11" t="n">
+      <c r="T11" t="n">
         <v>84</v>
       </c>
-      <c r="N11" t="n">
-        <v>86</v>
-      </c>
-      <c r="O11" t="n">
+      <c r="U11" t="n">
+        <v>80</v>
+      </c>
+      <c r="V11" t="n">
+        <v>58</v>
+      </c>
+      <c r="W11" t="n">
+        <v>73</v>
+      </c>
+      <c r="X11" t="n">
+        <v>100</v>
+      </c>
+      <c r="Y11" t="n">
         <v>79</v>
       </c>
-      <c r="P11" t="n">
-        <v>81</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>83</v>
-      </c>
-      <c r="R11" t="n">
-        <v>81</v>
-      </c>
-      <c r="S11" t="n">
-        <v>83</v>
-      </c>
-      <c r="T11" t="n">
-        <v>85</v>
-      </c>
-      <c r="U11" t="n">
-        <v>84</v>
-      </c>
-      <c r="V11" t="n">
-        <v>86</v>
-      </c>
-      <c r="W11" t="n">
-        <v>88</v>
-      </c>
-      <c r="X11" t="n">
-        <v>82</v>
-      </c>
-      <c r="Y11" t="n">
-        <v>84</v>
-      </c>
       <c r="Z11" t="n">
-        <v>86</v>
+        <v>67</v>
       </c>
       <c r="AA11" t="n">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="AB11" t="n">
-        <v>82</v>
-      </c>
-      <c r="AC11" t="n">
-        <v>84</v>
-      </c>
-      <c r="AD11" t="n">
-        <v>83.8</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>